<commit_message>
Frontend test report updated
</commit_message>
<xml_diff>
--- a/testing/docs/frontend/NeuChess_TesztJegyzokonyv_frontend.xlsx
+++ b/testing/docs/frontend/NeuChess_TesztJegyzokonyv_frontend.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oláh Ádám\Desktop\NeuChessHu\testing\docs\frontend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oláh Ádám\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BB4536F-25DD-4361-9BA5-54BA481A24B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3E3E0D-D944-40BE-BD89-8DFBD904F3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="167">
   <si>
     <t>Teszt azonosító</t>
   </si>
@@ -67,6 +67,9 @@
     <t>A NeuChess logó minden publikus oldalon látható.</t>
   </si>
   <si>
+    <t>Baranyai Gábor</t>
+  </si>
+  <si>
     <t>TC-003</t>
   </si>
   <si>
@@ -79,6 +82,12 @@
     <t>TC-004</t>
   </si>
   <si>
+    <t>Téma váltás dark/light</t>
+  </si>
+  <si>
+    <t>A téma gomb váltja az oldal színvilágát.</t>
+  </si>
+  <si>
     <t>TC-005</t>
   </si>
   <si>
@@ -151,6 +160,12 @@
     <t>TC-013</t>
   </si>
   <si>
+    <t>Bejelentkezés hálózati hiba</t>
+  </si>
+  <si>
+    <t>Hálózati hiba esetén általános hibaüzenet jelenik meg.</t>
+  </si>
+  <si>
     <t>TC-014</t>
   </si>
   <si>
@@ -163,9 +178,21 @@
     <t>TC-015</t>
   </si>
   <si>
+    <t>Sikeres bejelentkezés adminként</t>
+  </si>
+  <si>
+    <t>Admin szerepkörrel admin oldalra navigál.</t>
+  </si>
+  <si>
     <t>TC-016</t>
   </si>
   <si>
+    <t>redirect_uri kezelése login során</t>
+  </si>
+  <si>
+    <t>redirect_uri paraméter esetén OAuth close URL hívódik.</t>
+  </si>
+  <si>
     <t>TC-017</t>
   </si>
   <si>
@@ -178,138 +205,309 @@
     <t>TC-018</t>
   </si>
   <si>
+    <t>Regisztráció 1. lépés email validáció</t>
+  </si>
+  <si>
+    <t>Hibás emailnél nem aktív a továbblépés.</t>
+  </si>
+  <si>
     <t>TC-019</t>
   </si>
   <si>
+    <t>Regisztráció 1. lépés jelszó erősség</t>
+  </si>
+  <si>
+    <t>Gyenge jelszónál validációs hiba jelenik meg.</t>
+  </si>
+  <si>
     <t>TC-020</t>
   </si>
   <si>
+    <t>Regisztráció 1. lépés jelszó megerősítés</t>
+  </si>
+  <si>
+    <t>Nem egyező jelszavaknál hiba látható.</t>
+  </si>
+  <si>
     <t>TC-021</t>
   </si>
   <si>
+    <t>Regisztráció 1. lépés sikeres továbblépés</t>
+  </si>
+  <si>
+    <t>Érvényes adatokkal 2. lépésre navigál.</t>
+  </si>
+  <si>
     <t>TC-022</t>
   </si>
   <si>
+    <t>Stepper 2. lépés tiltás hiányos 1. lépésnél</t>
+  </si>
+  <si>
+    <t>A 2. lépés csak érvényes 1. lépés után kattintható.</t>
+  </si>
+  <si>
     <t>TC-023</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés nickname kötelező</t>
+  </si>
+  <si>
     <t>TC-024</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés nickname szabályok</t>
+  </si>
+  <si>
+    <t>Tiltott vagy túl rövid formátumot elutasít.</t>
+  </si>
+  <si>
     <t>TC-025</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés opcionális keresztnév</t>
+  </si>
+  <si>
+    <t>Üres keresztnév engedélyezett.</t>
+  </si>
+  <si>
     <t>TC-026</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés opcionális vezetéknév</t>
+  </si>
+  <si>
+    <t>Üres vezetéknév engedélyezett.</t>
+  </si>
+  <si>
     <t>TC-027</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés régió kiválasztás</t>
+  </si>
+  <si>
+    <t>A kiválasztott régió mentésre kerül.</t>
+  </si>
+  <si>
     <t>TC-028</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés születési dátum validáció</t>
+  </si>
+  <si>
+    <t>Jövőbeli dátum megadása tiltott.</t>
+  </si>
+  <si>
     <t>TC-029</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés Előző gomb</t>
+  </si>
+  <si>
+    <t>Visszalépéskor az addig kitöltött adatok megmaradnak.</t>
+  </si>
+  <si>
     <t>TC-030</t>
   </si>
   <si>
+    <t>Regisztráció 2. lépés Következő gomb</t>
+  </si>
+  <si>
+    <t>Érvényes adatokkal 3. lépésre navigál.</t>
+  </si>
+  <si>
+    <t>TC-031</t>
+  </si>
+  <si>
+    <t>Stepper 3. lépés tiltás hiányos 2. lépésnél</t>
+  </si>
+  <si>
+    <t>A 3. lépés csak kitöltött nickname után kattintható.</t>
+  </si>
+  <si>
+    <t>TC-032</t>
+  </si>
+  <si>
+    <t>Regisztráció 3. lépés összegző adatok</t>
+  </si>
+  <si>
+    <t>A megadott email és profiladatok helyesen jelennek meg.</t>
+  </si>
+  <si>
+    <t>TC-033</t>
+  </si>
+  <si>
+    <t>Regisztráció 3. lépés ÁSZF kötelező</t>
+  </si>
+  <si>
+    <t>ÁSZF elfogadás nélkül nincs sikeres beküldés.</t>
+  </si>
+  <si>
+    <t>TC-034</t>
+  </si>
+  <si>
+    <t>Regisztráció 3. lépés ÁSZF link</t>
+  </si>
+  <si>
+    <t>A link új lapon nyílik locale-függő URL-re.</t>
+  </si>
+  <si>
+    <t>TC-035</t>
+  </si>
+  <si>
+    <t>Regisztráció 3. lépés szerver hiba</t>
+  </si>
+  <si>
+    <t>API hiba esetén backend üzenet vagy fallback hiba jelenik meg.</t>
+  </si>
+  <si>
+    <t>TC-036</t>
+  </si>
+  <si>
     <t>Regisztráció sikeres befejezés</t>
   </si>
   <si>
     <t>Siker után automatikusan beléptet és profilra visz.</t>
   </si>
   <si>
+    <t>TC-037</t>
+  </si>
+  <si>
     <t>Regisztráció adatok resetje siker után</t>
   </si>
   <si>
     <t>Sikeres regisztráció után a store adatai ürülnek.</t>
   </si>
   <si>
+    <t>TC-038</t>
+  </si>
+  <si>
     <t>Dinamikus user route betöltés</t>
   </si>
   <si>
     <t>A /user/:nickname oldal a megfelelő profilt tölti be.</t>
   </si>
   <si>
+    <t>TC-039</t>
+  </si>
+  <si>
     <t>Profil oldal cím frissítése</t>
   </si>
   <si>
     <t>A böngészőfül címe a nickname-re vált.</t>
   </si>
   <si>
+    <t>TC-040</t>
+  </si>
+  <si>
     <t>Profil statisztika panel megjelenése</t>
   </si>
   <si>
     <t>Personal stat panel helyesen renderelődik.</t>
   </si>
   <si>
+    <t>TC-041</t>
+  </si>
+  <si>
     <t>Meccs információk panel megjelenése</t>
   </si>
   <si>
     <t>Match infos panel megjelenik és adatot mutat.</t>
   </si>
   <si>
+    <t>TC-042</t>
+  </si>
+  <si>
     <t>Sakk statisztika panel megjelenése</t>
   </si>
   <si>
     <t>Chess stat panel megjelenik és adatot mutat.</t>
   </si>
   <si>
+    <t>TC-043</t>
+  </si>
+  <si>
     <t>Saját profil szerkesztés engedélyezés</t>
   </si>
   <si>
     <t>Tulajdonosként a profilmezők szerkeszthetők.</t>
   </si>
   <si>
+    <t>TC-044</t>
+  </si>
+  <si>
     <t>Idegen profil szerkesztés tiltás</t>
   </si>
   <si>
     <t>Nem tulajdonosként szerkesztés nem érhető el.</t>
   </si>
   <si>
+    <t>TC-045</t>
+  </si>
+  <si>
     <t>Profil mentés</t>
   </si>
   <si>
     <t>Mentés után új adatok töltődnek vissza a felületen.</t>
   </si>
   <si>
+    <t>TC-046</t>
+  </si>
+  <si>
     <t>Profil törlés saját fiókkal</t>
   </si>
   <si>
     <t>Saját fiók törlése után kijelentkezik és sign inre visz.</t>
   </si>
   <si>
+    <t>TC-047</t>
+  </si>
+  <si>
     <t>Logout gomb működése</t>
   </si>
   <si>
     <t>Kijelentkezés törli a session adatokat és visszairányít.</t>
   </si>
   <si>
+    <t>TC-048</t>
+  </si>
+  <si>
     <t>Admin oldal elérhetősége adminnak</t>
   </si>
   <si>
     <t>Adminként az admin lista oldal betöltődik.</t>
   </si>
   <si>
+    <t>TC-049</t>
+  </si>
+  <si>
     <t>Admin user lista megjelenítés</t>
   </si>
   <si>
     <t>A felhasználói kártyák listázása működik.</t>
   </si>
   <si>
+    <t>TC-050</t>
+  </si>
+  <si>
     <t>Admin szerkesztés felhasználón</t>
   </si>
   <si>
     <t>Admin mentés frissíti az adott felhasználó kártyáját.</t>
   </si>
   <si>
+    <t>TC-051</t>
+  </si>
+  <si>
     <t>Admin törlés felhasználón</t>
   </si>
   <si>
     <t>Admin törlés után a törölt user eltűnik a listából.</t>
   </si>
   <si>
+    <t>TC-052</t>
+  </si>
+  <si>
     <t>Oldalcím lokalizált route-okon</t>
   </si>
   <si>
@@ -317,6 +515,9 @@
   </si>
   <si>
     <t>Sikeres</t>
+  </si>
+  <si>
+    <t>Üres 'nickname' esetén validációs hiba jelenik meg.</t>
   </si>
   <si>
     <t>Téma mentés localStorage-ban</t>
@@ -422,7 +623,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,22 +643,22 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -473,24 +674,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -828,7 +1011,7 @@
         <v>46139</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -851,18 +1034,18 @@
         <v>46139</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D4" s="15" t="s">
         <v>10</v>
@@ -874,18 +1057,18 @@
         <v>46139</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>99</v>
+        <v>166</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>10</v>
@@ -897,18 +1080,18 @@
         <v>46139</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>10</v>
@@ -920,18 +1103,18 @@
         <v>46139</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>10</v>
@@ -943,18 +1126,18 @@
         <v>46139</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>10</v>
@@ -966,18 +1149,18 @@
         <v>46139</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>10</v>
@@ -989,18 +1172,18 @@
         <v>46139</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D10" s="15" t="s">
         <v>10</v>
@@ -1012,18 +1195,18 @@
         <v>46139</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>10</v>
@@ -1035,18 +1218,18 @@
         <v>46139</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D12" s="15" t="s">
         <v>10</v>
@@ -1058,18 +1241,18 @@
         <v>46139</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>10</v>
@@ -1081,18 +1264,18 @@
         <v>46139</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>10</v>
@@ -1104,18 +1287,18 @@
         <v>46139</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>64</v>
+        <v>114</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>65</v>
+        <v>115</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>10</v>
@@ -1127,18 +1310,18 @@
         <v>46139</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>66</v>
+        <v>117</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>67</v>
+        <v>118</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>10</v>
@@ -1150,18 +1333,18 @@
         <v>46139</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>69</v>
+        <v>121</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>10</v>
@@ -1173,18 +1356,18 @@
         <v>46139</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>70</v>
+        <v>123</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>71</v>
+        <v>124</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>10</v>
@@ -1196,18 +1379,18 @@
         <v>46139</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>72</v>
+        <v>126</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>73</v>
+        <v>127</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>10</v>
@@ -1219,18 +1402,18 @@
         <v>46139</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B20" s="13" t="s">
-        <v>74</v>
+        <v>129</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>10</v>
@@ -1242,18 +1425,18 @@
         <v>46139</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>76</v>
+        <v>132</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>77</v>
+        <v>133</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>10</v>
@@ -1265,18 +1448,18 @@
         <v>46139</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="B22" s="13" t="s">
-        <v>78</v>
+        <v>135</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>79</v>
+        <v>136</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>10</v>
@@ -1288,18 +1471,18 @@
         <v>46139</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>80</v>
+        <v>138</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>81</v>
+        <v>139</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>10</v>
@@ -1311,18 +1494,18 @@
         <v>46139</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>82</v>
+        <v>141</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>83</v>
+        <v>142</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>10</v>
@@ -1334,18 +1517,18 @@
         <v>46139</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>84</v>
+        <v>144</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>85</v>
+        <v>145</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>10</v>
@@ -1357,18 +1540,18 @@
         <v>46139</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>86</v>
+        <v>147</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>87</v>
+        <v>148</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>10</v>
@@ -1380,18 +1563,18 @@
         <v>46139</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>88</v>
+        <v>150</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>89</v>
+        <v>151</v>
       </c>
       <c r="D27" s="9" t="s">
         <v>10</v>
@@ -1403,18 +1586,18 @@
         <v>46139</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>60</v>
+        <v>86</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>90</v>
+        <v>153</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>91</v>
+        <v>154</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>10</v>
@@ -1426,18 +1609,18 @@
         <v>46139</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>92</v>
+        <v>156</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>93</v>
+        <v>157</v>
       </c>
       <c r="D29" s="9" t="s">
         <v>10</v>
@@ -1449,18 +1632,18 @@
         <v>46139</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>94</v>
+        <v>159</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>95</v>
+        <v>160</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>10</v>
@@ -1472,229 +1655,537 @@
         <v>46139</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>98</v>
+        <v>164</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>63</v>
+        <v>95</v>
       </c>
       <c r="B31" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F33" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F35" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G37" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F39" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C42" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G42" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C46" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F46" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F47" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B48" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="C31" s="12" t="s">
+      <c r="C48" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" s="10">
-        <v>46139</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="18"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="23"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="18"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="23"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="18"/>
-      <c r="B34" s="19"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="23"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="18"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="23"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="18"/>
-      <c r="B36" s="19"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="23"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="18"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="22"/>
-      <c r="G37" s="23"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="18"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="22"/>
-      <c r="G38" s="23"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="18"/>
-      <c r="B39" s="19"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="21"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="22"/>
-      <c r="G39" s="23"/>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="18"/>
-      <c r="B40" s="19"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="23"/>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="18"/>
-      <c r="B41" s="19"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="21"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="23"/>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="18"/>
-      <c r="B42" s="19"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="21"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="23"/>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="18"/>
-      <c r="B43" s="19"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="21"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="23"/>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="18"/>
-      <c r="B44" s="19"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="23"/>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="18"/>
-      <c r="B45" s="19"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="21"/>
-      <c r="E45" s="18"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="23"/>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="18"/>
-      <c r="B46" s="19"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="18"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="23"/>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="18"/>
-      <c r="B47" s="19"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="21"/>
-      <c r="E47" s="18"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="23"/>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="18"/>
-      <c r="B48" s="19"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="18"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="23"/>
+      <c r="D48" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F48" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="18"/>
-      <c r="B49" s="19"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="21"/>
-      <c r="E49" s="18"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="23"/>
+      <c r="A49" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F49" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="18"/>
-      <c r="B50" s="19"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="21"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="23"/>
+      <c r="A50" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F50" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="18"/>
-      <c r="B51" s="19"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="21"/>
-      <c r="E51" s="18"/>
-      <c r="F51" s="22"/>
-      <c r="G51" s="23"/>
+      <c r="A51" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F51" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="18"/>
-      <c r="B52" s="19"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="21"/>
-      <c r="E52" s="18"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="23"/>
+      <c r="A52" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="D52" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F52" s="17">
+        <v>46139</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="18"/>
-      <c r="B53" s="19"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="21"/>
-      <c r="E53" s="18"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="23"/>
+      <c r="A53" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F53" s="10">
+        <v>46139</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>164</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>